<commit_message>
moved some code and updated for newest batch
</commit_message>
<xml_diff>
--- a/apcd_export_import/apcd_source_tables.xlsx
+++ b/apcd_export_import/apcd_source_tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwhitehurst.KC\OneDrive - King County\Documents\R\claims_data\apcd_export_import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96D94B5B-C88F-49AF-93B7-98695E349A80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCDC27D2-C05A-4E85-9924-3EB4CCEA0E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4860" yWindow="3600" windowWidth="38535" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="174">
   <si>
     <t>claims</t>
   </si>
@@ -552,6 +552,12 @@
   </si>
   <si>
     <t>apcd_dental_claim</t>
+  </si>
+  <si>
+    <t>apcd_claim_bh</t>
+  </si>
+  <si>
+    <t>stage_apcd_claim_bh</t>
   </si>
 </sst>
 </file>
@@ -869,7 +875,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D87"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
@@ -911,13 +917,13 @@
         <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C3" t="s">
         <v>71</v>
       </c>
       <c r="D3" t="s">
-        <v>128</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -925,13 +931,13 @@
         <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>151</v>
+        <v>171</v>
       </c>
       <c r="C4" t="s">
         <v>71</v>
       </c>
       <c r="D4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -939,13 +945,13 @@
         <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C5" t="s">
         <v>71</v>
       </c>
       <c r="D5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -953,13 +959,13 @@
         <v>55</v>
       </c>
       <c r="B6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C6" t="s">
         <v>71</v>
       </c>
       <c r="D6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -967,13 +973,13 @@
         <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>153</v>
       </c>
       <c r="C7" t="s">
         <v>71</v>
       </c>
       <c r="D7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -981,13 +987,13 @@
         <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>154</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s">
         <v>71</v>
       </c>
       <c r="D8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -995,13 +1001,13 @@
         <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C9" t="s">
         <v>71</v>
       </c>
       <c r="D9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1009,13 +1015,13 @@
         <v>55</v>
       </c>
       <c r="B10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C10" t="s">
         <v>71</v>
       </c>
       <c r="D10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1023,13 +1029,13 @@
         <v>55</v>
       </c>
       <c r="B11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C11" t="s">
         <v>71</v>
       </c>
       <c r="D11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1037,13 +1043,13 @@
         <v>55</v>
       </c>
       <c r="B12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C12" t="s">
         <v>71</v>
       </c>
       <c r="D12" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1051,13 +1057,13 @@
         <v>55</v>
       </c>
       <c r="B13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C13" t="s">
         <v>71</v>
       </c>
       <c r="D13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1065,13 +1071,13 @@
         <v>55</v>
       </c>
       <c r="B14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C14" t="s">
         <v>71</v>
       </c>
       <c r="D14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1079,13 +1085,13 @@
         <v>55</v>
       </c>
       <c r="B15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C15" t="s">
         <v>71</v>
       </c>
       <c r="D15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1093,13 +1099,13 @@
         <v>55</v>
       </c>
       <c r="B16" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C16" t="s">
         <v>71</v>
       </c>
       <c r="D16" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1107,13 +1113,13 @@
         <v>55</v>
       </c>
       <c r="B17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C17" t="s">
         <v>71</v>
       </c>
       <c r="D17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1121,13 +1127,13 @@
         <v>55</v>
       </c>
       <c r="B18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C18" t="s">
         <v>71</v>
       </c>
       <c r="D18" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1135,13 +1141,13 @@
         <v>55</v>
       </c>
       <c r="B19" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C19" t="s">
         <v>71</v>
       </c>
       <c r="D19" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1149,13 +1155,13 @@
         <v>55</v>
       </c>
       <c r="B20" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C20" t="s">
         <v>71</v>
       </c>
       <c r="D20" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1163,13 +1169,13 @@
         <v>55</v>
       </c>
       <c r="B21" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C21" t="s">
         <v>71</v>
       </c>
       <c r="D21" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -1177,13 +1183,13 @@
         <v>55</v>
       </c>
       <c r="B22" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C22" t="s">
         <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1191,13 +1197,13 @@
         <v>55</v>
       </c>
       <c r="B23" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
       </c>
       <c r="D23" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1205,27 +1211,27 @@
         <v>55</v>
       </c>
       <c r="B24" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C24" t="s">
         <v>71</v>
       </c>
       <c r="D24" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="B25" t="s">
-        <v>1</v>
+        <v>170</v>
       </c>
       <c r="C25" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="D25" t="s">
-        <v>73</v>
+        <v>149</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1233,13 +1239,13 @@
         <v>0</v>
       </c>
       <c r="B26" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C26" t="s">
         <v>52</v>
       </c>
       <c r="D26" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1247,13 +1253,13 @@
         <v>0</v>
       </c>
       <c r="B27" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C27" t="s">
         <v>52</v>
       </c>
       <c r="D27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1261,13 +1267,13 @@
         <v>0</v>
       </c>
       <c r="B28" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C28" t="s">
         <v>52</v>
       </c>
       <c r="D28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1275,13 +1281,13 @@
         <v>0</v>
       </c>
       <c r="B29" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C29" t="s">
         <v>52</v>
       </c>
       <c r="D29" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1289,13 +1295,13 @@
         <v>0</v>
       </c>
       <c r="B30" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C30" t="s">
         <v>52</v>
       </c>
       <c r="D30" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1303,13 +1309,13 @@
         <v>0</v>
       </c>
       <c r="B31" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C31" t="s">
         <v>52</v>
       </c>
       <c r="D31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1317,13 +1323,13 @@
         <v>0</v>
       </c>
       <c r="B32" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C32" t="s">
         <v>52</v>
       </c>
       <c r="D32" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1331,13 +1337,13 @@
         <v>0</v>
       </c>
       <c r="B33" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C33" t="s">
         <v>52</v>
       </c>
       <c r="D33" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1345,13 +1351,13 @@
         <v>0</v>
       </c>
       <c r="B34" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C34" t="s">
         <v>52</v>
       </c>
       <c r="D34" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -1359,13 +1365,13 @@
         <v>0</v>
       </c>
       <c r="B35" t="s">
-        <v>62</v>
+        <v>10</v>
       </c>
       <c r="C35" t="s">
         <v>52</v>
       </c>
       <c r="D35" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -1373,13 +1379,13 @@
         <v>0</v>
       </c>
       <c r="B36" t="s">
-        <v>11</v>
+        <v>62</v>
       </c>
       <c r="C36" t="s">
         <v>52</v>
       </c>
       <c r="D36" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1387,13 +1393,13 @@
         <v>0</v>
       </c>
       <c r="B37" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C37" t="s">
         <v>52</v>
       </c>
       <c r="D37" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1401,13 +1407,13 @@
         <v>0</v>
       </c>
       <c r="B38" t="s">
-        <v>63</v>
+        <v>12</v>
       </c>
       <c r="C38" t="s">
         <v>52</v>
       </c>
       <c r="D38" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1415,13 +1421,13 @@
         <v>0</v>
       </c>
       <c r="B39" t="s">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="C39" t="s">
         <v>52</v>
       </c>
       <c r="D39" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -1429,13 +1435,13 @@
         <v>0</v>
       </c>
       <c r="B40" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C40" t="s">
         <v>52</v>
       </c>
       <c r="D40" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1443,13 +1449,13 @@
         <v>0</v>
       </c>
       <c r="B41" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C41" t="s">
         <v>52</v>
       </c>
       <c r="D41" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1457,13 +1463,13 @@
         <v>0</v>
       </c>
       <c r="B42" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C42" t="s">
         <v>52</v>
       </c>
       <c r="D42" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1471,13 +1477,13 @@
         <v>0</v>
       </c>
       <c r="B43" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C43" t="s">
         <v>52</v>
       </c>
       <c r="D43" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1485,13 +1491,13 @@
         <v>0</v>
       </c>
       <c r="B44" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C44" t="s">
         <v>52</v>
       </c>
       <c r="D44" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1499,13 +1505,13 @@
         <v>0</v>
       </c>
       <c r="B45" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C45" t="s">
         <v>52</v>
       </c>
       <c r="D45" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -1513,13 +1519,13 @@
         <v>0</v>
       </c>
       <c r="B46" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C46" t="s">
         <v>52</v>
       </c>
       <c r="D46" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -1527,13 +1533,13 @@
         <v>0</v>
       </c>
       <c r="B47" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C47" t="s">
         <v>52</v>
       </c>
       <c r="D47" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1541,13 +1547,13 @@
         <v>0</v>
       </c>
       <c r="B48" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C48" t="s">
         <v>52</v>
       </c>
       <c r="D48" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1555,13 +1561,13 @@
         <v>0</v>
       </c>
       <c r="B49" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C49" t="s">
         <v>52</v>
       </c>
       <c r="D49" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1569,13 +1575,13 @@
         <v>0</v>
       </c>
       <c r="B50" t="s">
-        <v>64</v>
+        <v>23</v>
       </c>
       <c r="C50" t="s">
         <v>52</v>
       </c>
       <c r="D50" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -1583,13 +1589,13 @@
         <v>0</v>
       </c>
       <c r="B51" t="s">
-        <v>24</v>
+        <v>64</v>
       </c>
       <c r="C51" t="s">
         <v>52</v>
       </c>
       <c r="D51" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -1597,13 +1603,13 @@
         <v>0</v>
       </c>
       <c r="B52" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C52" t="s">
         <v>52</v>
       </c>
       <c r="D52" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -1611,13 +1617,13 @@
         <v>0</v>
       </c>
       <c r="B53" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C53" t="s">
         <v>52</v>
       </c>
       <c r="D53" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -1625,13 +1631,13 @@
         <v>0</v>
       </c>
       <c r="B54" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C54" t="s">
         <v>52</v>
       </c>
       <c r="D54" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -1639,13 +1645,13 @@
         <v>0</v>
       </c>
       <c r="B55" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C55" t="s">
         <v>52</v>
       </c>
       <c r="D55" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -1653,13 +1659,13 @@
         <v>0</v>
       </c>
       <c r="B56" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C56" t="s">
         <v>52</v>
       </c>
       <c r="D56" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -1667,13 +1673,13 @@
         <v>0</v>
       </c>
       <c r="B57" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C57" t="s">
         <v>52</v>
       </c>
       <c r="D57" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -1681,13 +1687,13 @@
         <v>0</v>
       </c>
       <c r="B58" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C58" t="s">
         <v>52</v>
       </c>
       <c r="D58" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -1695,13 +1701,13 @@
         <v>0</v>
       </c>
       <c r="B59" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C59" t="s">
         <v>52</v>
       </c>
       <c r="D59" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -1709,13 +1715,13 @@
         <v>0</v>
       </c>
       <c r="B60" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C60" t="s">
         <v>52</v>
       </c>
       <c r="D60" t="s">
-        <v>60</v>
+        <v>107</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -1723,13 +1729,13 @@
         <v>0</v>
       </c>
       <c r="B61" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C61" t="s">
         <v>52</v>
       </c>
       <c r="D61" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -1737,13 +1743,13 @@
         <v>0</v>
       </c>
       <c r="B62" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C62" t="s">
         <v>52</v>
       </c>
       <c r="D62" t="s">
-        <v>108</v>
+        <v>61</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -1751,13 +1757,13 @@
         <v>0</v>
       </c>
       <c r="B63" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C63" t="s">
         <v>52</v>
       </c>
       <c r="D63" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -1765,13 +1771,13 @@
         <v>0</v>
       </c>
       <c r="B64" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="C64" t="s">
         <v>52</v>
       </c>
       <c r="D64" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -1779,13 +1785,13 @@
         <v>0</v>
       </c>
       <c r="B65" t="s">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="C65" t="s">
         <v>52</v>
       </c>
       <c r="D65" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -1793,13 +1799,13 @@
         <v>0</v>
       </c>
       <c r="B66" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C66" t="s">
         <v>52</v>
       </c>
       <c r="D66" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -1807,13 +1813,13 @@
         <v>0</v>
       </c>
       <c r="B67" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C67" t="s">
         <v>52</v>
       </c>
       <c r="D67" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -1821,13 +1827,13 @@
         <v>0</v>
       </c>
       <c r="B68" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C68" t="s">
         <v>52</v>
       </c>
       <c r="D68" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -1835,13 +1841,13 @@
         <v>0</v>
       </c>
       <c r="B69" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C69" t="s">
         <v>52</v>
       </c>
       <c r="D69" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -1849,13 +1855,13 @@
         <v>0</v>
       </c>
       <c r="B70" t="s">
-        <v>66</v>
+        <v>41</v>
       </c>
       <c r="C70" t="s">
         <v>52</v>
       </c>
       <c r="D70" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -1863,13 +1869,13 @@
         <v>0</v>
       </c>
       <c r="B71" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="C71" t="s">
         <v>52</v>
       </c>
       <c r="D71" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -1877,13 +1883,13 @@
         <v>0</v>
       </c>
       <c r="B72" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C72" t="s">
         <v>52</v>
       </c>
       <c r="D72" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -1891,13 +1897,13 @@
         <v>0</v>
       </c>
       <c r="B73" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C73" t="s">
         <v>52</v>
       </c>
       <c r="D73" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -1905,13 +1911,13 @@
         <v>0</v>
       </c>
       <c r="B74" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C74" t="s">
         <v>52</v>
       </c>
       <c r="D74" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -1919,13 +1925,13 @@
         <v>0</v>
       </c>
       <c r="B75" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C75" t="s">
         <v>52</v>
       </c>
       <c r="D75" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -1933,13 +1939,13 @@
         <v>0</v>
       </c>
       <c r="B76" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C76" t="s">
         <v>52</v>
       </c>
       <c r="D76" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -1947,13 +1953,13 @@
         <v>0</v>
       </c>
       <c r="B77" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C77" t="s">
         <v>52</v>
       </c>
       <c r="D77" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -1961,13 +1967,13 @@
         <v>0</v>
       </c>
       <c r="B78" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C78" t="s">
         <v>52</v>
       </c>
       <c r="D78" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -1975,13 +1981,13 @@
         <v>0</v>
       </c>
       <c r="B79" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C79" t="s">
         <v>52</v>
       </c>
       <c r="D79" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -1989,27 +1995,27 @@
         <v>0</v>
       </c>
       <c r="B80" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C80" t="s">
         <v>52</v>
       </c>
       <c r="D80" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="B81" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C81" t="s">
         <v>52</v>
       </c>
       <c r="D81" t="s">
-        <v>53</v>
+        <v>126</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -2017,27 +2023,27 @@
         <v>52</v>
       </c>
       <c r="B82" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C82" t="s">
         <v>52</v>
       </c>
       <c r="D82" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B83" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C83" t="s">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="D83" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -2045,13 +2051,13 @@
         <v>55</v>
       </c>
       <c r="B84" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C84" t="s">
         <v>72</v>
       </c>
       <c r="D84" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -2059,13 +2065,13 @@
         <v>55</v>
       </c>
       <c r="B85" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C85" t="s">
         <v>72</v>
       </c>
       <c r="D85" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -2073,13 +2079,13 @@
         <v>55</v>
       </c>
       <c r="B86" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C86" t="s">
         <v>72</v>
       </c>
       <c r="D86" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -2087,12 +2093,26 @@
         <v>55</v>
       </c>
       <c r="B87" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C87" t="s">
         <v>72</v>
       </c>
       <c r="D87" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>55</v>
+      </c>
+      <c r="B88" t="s">
+        <v>61</v>
+      </c>
+      <c r="C88" t="s">
+        <v>72</v>
+      </c>
+      <c r="D88" t="s">
         <v>61</v>
       </c>
     </row>

</xml_diff>